<commit_message>
Added csv data for link quality testing between dalplex and goldberg
</commit_message>
<xml_diff>
--- a/data/PlexToGB/all.xlsx
+++ b/data/PlexToGB/all.xlsx
@@ -1,27 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Jon/usra2026/data/PlexToGB/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{28ACBBD6-38CE-2E4F-B626-39EE4EF9C53D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EA48FE6-F70F-2E46-B163-A8C5A81635CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="1000" windowWidth="27640" windowHeight="16440" activeTab="1" xr2:uid="{7BF87952-EAF1-3342-A433-EE12F1C9EE04}"/>
+    <workbookView xWindow="780" yWindow="1000" windowWidth="27640" windowHeight="16440" xr2:uid="{7BF87952-EAF1-3342-A433-EE12F1C9EE04}"/>
   </bookViews>
   <sheets>
     <sheet name="all" sheetId="1" r:id="rId1"/>
     <sheet name="Final Results" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -1526,16 +1539,14 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="33" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="18" fillId="34" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
@@ -1920,84 +1931,82 @@
     <col min="2" max="2" width="13.83203125" customWidth="1"/>
     <col min="3" max="3" width="11.83203125" customWidth="1"/>
     <col min="4" max="4" width="13.5" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" style="4"/>
     <col min="8" max="8" width="10.83203125" style="2"/>
     <col min="13" max="13" width="10.83203125" style="3"/>
-    <col min="20" max="20" width="10.83203125" style="4"/>
     <col min="21" max="21" width="10.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" s="5" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:27" s="4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
         <v>230</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>231</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>232</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="4" t="s">
         <v>234</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="4" t="s">
         <v>235</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="G1" s="4" t="s">
         <v>316</v>
       </c>
-      <c r="H1" s="9"/>
-      <c r="I1" s="5" t="s">
+      <c r="H1" s="7"/>
+      <c r="I1" s="4" t="s">
         <v>315</v>
       </c>
-      <c r="J1" s="6" t="s">
+      <c r="J1" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="K1" s="4" t="s">
         <v>235</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="L1" s="4" t="s">
         <v>234</v>
       </c>
-      <c r="M1" s="10"/>
-      <c r="N1" s="5" t="s">
+      <c r="M1" s="8"/>
+      <c r="N1" s="4" t="s">
         <v>230</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="O1" s="4" t="s">
         <v>314</v>
       </c>
-      <c r="P1" s="5" t="s">
+      <c r="P1" s="4" t="s">
         <v>232</v>
       </c>
-      <c r="Q1" s="5" t="s">
+      <c r="Q1" s="4" t="s">
         <v>233</v>
       </c>
-      <c r="R1" s="6" t="s">
+      <c r="R1" s="5" t="s">
         <v>234</v>
       </c>
-      <c r="S1" s="5" t="s">
+      <c r="S1" s="4" t="s">
         <v>235</v>
       </c>
-      <c r="T1" s="8" t="s">
+      <c r="T1" s="4" t="s">
         <v>316</v>
       </c>
-      <c r="U1" s="9"/>
-      <c r="V1" s="5" t="s">
+      <c r="U1" s="7"/>
+      <c r="V1" s="4" t="s">
         <v>232</v>
       </c>
-      <c r="W1" s="6" t="s">
+      <c r="W1" s="5" t="s">
         <v>233</v>
       </c>
-      <c r="X1" s="5" t="s">
+      <c r="X1" s="4" t="s">
         <v>234</v>
       </c>
-      <c r="Y1" s="5" t="s">
+      <c r="Y1" s="4" t="s">
         <v>235</v>
       </c>
-      <c r="AA1" s="6"/>
+      <c r="AA1" s="5"/>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A2">
@@ -2018,7 +2027,7 @@
       <c r="F2">
         <v>-14.75</v>
       </c>
-      <c r="G2" s="4">
+      <c r="G2">
         <f>D2-B2</f>
         <v>2.9821000099182129</v>
       </c>
@@ -2052,7 +2061,7 @@
       <c r="S2">
         <v>-5.75</v>
       </c>
-      <c r="T2" s="4">
+      <c r="T2">
         <f>Q2-O2</f>
         <v>3.078279972076416</v>
       </c>
@@ -2089,7 +2098,7 @@
       <c r="F3">
         <v>-14.25</v>
       </c>
-      <c r="G3" s="4">
+      <c r="G3">
         <f>D3-B3</f>
         <v>4.109260082244873</v>
       </c>
@@ -2117,7 +2126,7 @@
       <c r="S3">
         <v>-15</v>
       </c>
-      <c r="T3" s="4">
+      <c r="T3">
         <f>Q3-O3</f>
         <v>12.026700019836426</v>
       </c>
@@ -2154,7 +2163,7 @@
       <c r="F4">
         <v>-12.75</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4">
         <f>D4-B4</f>
         <v>10.206660032272339</v>
       </c>
@@ -2188,7 +2197,7 @@
       <c r="S4">
         <v>-14.75</v>
       </c>
-      <c r="T4" s="4">
+      <c r="T4">
         <f>Q4-O4</f>
         <v>6.8313801288604736</v>
       </c>
@@ -2225,7 +2234,7 @@
       <c r="F5">
         <v>-11.75</v>
       </c>
-      <c r="G5" s="4">
+      <c r="G5">
         <f t="shared" ref="G5:G31" si="0">D5-B5</f>
         <v>18.20403003692627</v>
       </c>
@@ -2253,7 +2262,7 @@
       <c r="S5">
         <v>-10.25</v>
       </c>
-      <c r="T5" s="4">
+      <c r="T5">
         <f>Q5-O5</f>
         <v>12.067489862442017</v>
       </c>
@@ -2290,7 +2299,7 @@
       <c r="F6">
         <v>-9.75</v>
       </c>
-      <c r="G6" s="4">
+      <c r="G6">
         <f t="shared" si="0"/>
         <v>3.2466199398040771</v>
       </c>
@@ -2324,8 +2333,8 @@
       <c r="S6">
         <v>-16.5</v>
       </c>
-      <c r="T6" s="4">
-        <f t="shared" ref="T3:T66" si="1">Q6-O6</f>
+      <c r="T6">
+        <f t="shared" ref="T6:T66" si="1">Q6-O6</f>
         <v>3.1116800308227539</v>
       </c>
       <c r="V6">
@@ -2361,7 +2370,7 @@
       <c r="F7">
         <v>-15.75</v>
       </c>
-      <c r="G7" s="4">
+      <c r="G7">
         <f t="shared" si="0"/>
         <v>3.6383600234985352</v>
       </c>
@@ -2389,7 +2398,7 @@
       <c r="S7">
         <v>-16.75</v>
       </c>
-      <c r="T7" s="4">
+      <c r="T7">
         <f t="shared" si="1"/>
         <v>3.0944499969482422</v>
       </c>
@@ -2426,7 +2435,7 @@
       <c r="F8">
         <v>-18.5</v>
       </c>
-      <c r="G8" s="4">
+      <c r="G8">
         <f t="shared" si="0"/>
         <v>3.8204400539398193</v>
       </c>
@@ -2460,7 +2469,7 @@
       <c r="S8">
         <v>-17.25</v>
       </c>
-      <c r="T8" s="4">
+      <c r="T8">
         <f t="shared" si="1"/>
         <v>21.575010061264038</v>
       </c>
@@ -2496,7 +2505,7 @@
       <c r="F9">
         <v>-11.25</v>
       </c>
-      <c r="G9" s="4">
+      <c r="G9">
         <f t="shared" si="0"/>
         <v>2.8129599094390869</v>
       </c>
@@ -2524,7 +2533,7 @@
       <c r="S9">
         <v>-7.75</v>
       </c>
-      <c r="T9" s="4">
+      <c r="T9">
         <f t="shared" si="1"/>
         <v>22.435250043869019</v>
       </c>
@@ -2561,7 +2570,7 @@
       <c r="F10">
         <v>-10</v>
       </c>
-      <c r="G10" s="4">
+      <c r="G10">
         <f t="shared" si="0"/>
         <v>2.9275600910186768</v>
       </c>
@@ -2589,7 +2598,7 @@
       <c r="S10">
         <v>-7.25</v>
       </c>
-      <c r="T10" s="4">
+      <c r="T10">
         <f t="shared" si="1"/>
         <v>23.874329805374146</v>
       </c>
@@ -2626,7 +2635,7 @@
       <c r="F11">
         <v>-10.5</v>
       </c>
-      <c r="G11" s="4">
+      <c r="G11">
         <f t="shared" si="0"/>
         <v>10.228149890899658</v>
       </c>
@@ -2660,7 +2669,7 @@
       <c r="S11">
         <v>-12.5</v>
       </c>
-      <c r="T11" s="4">
+      <c r="T11">
         <f t="shared" si="1"/>
         <v>23.56466007232666</v>
       </c>
@@ -2691,7 +2700,7 @@
       <c r="F12">
         <v>-9.25</v>
       </c>
-      <c r="G12" s="4">
+      <c r="G12">
         <f t="shared" si="0"/>
         <v>3.525670051574707</v>
       </c>
@@ -2719,7 +2728,7 @@
       <c r="S12">
         <v>-7.5</v>
       </c>
-      <c r="T12" s="4">
+      <c r="T12">
         <f t="shared" si="1"/>
         <v>13.361680030822754</v>
       </c>
@@ -2756,7 +2765,7 @@
       <c r="F13">
         <v>-10.75</v>
       </c>
-      <c r="G13" s="4">
+      <c r="G13">
         <f t="shared" si="0"/>
         <v>10.636470079421997</v>
       </c>
@@ -2790,7 +2799,7 @@
       <c r="S13">
         <v>-13</v>
       </c>
-      <c r="T13" s="4">
+      <c r="T13">
         <f t="shared" si="1"/>
         <v>24.668970108032227</v>
       </c>
@@ -2821,7 +2830,7 @@
       <c r="F14">
         <v>-11.5</v>
       </c>
-      <c r="G14" s="4">
+      <c r="G14">
         <f t="shared" si="0"/>
         <v>3.6838400363922119</v>
       </c>
@@ -2849,7 +2858,7 @@
       <c r="S14">
         <v>-14.5</v>
       </c>
-      <c r="T14" s="4">
+      <c r="T14">
         <f t="shared" si="1"/>
         <v>7.6366498470306396</v>
       </c>
@@ -2880,7 +2889,7 @@
       <c r="F15">
         <v>-16.75</v>
       </c>
-      <c r="G15" s="4">
+      <c r="G15">
         <f t="shared" si="0"/>
         <v>18.143290042877197</v>
       </c>
@@ -2914,7 +2923,7 @@
       <c r="S15">
         <v>-13.5</v>
       </c>
-      <c r="T15" s="4">
+      <c r="T15">
         <f t="shared" si="1"/>
         <v>3.6272799968719482</v>
       </c>
@@ -2945,7 +2954,7 @@
       <c r="F16">
         <v>-12</v>
       </c>
-      <c r="G16" s="4">
+      <c r="G16">
         <f t="shared" si="0"/>
         <v>11.001420021057129</v>
       </c>
@@ -2973,7 +2982,7 @@
       <c r="S16">
         <v>-9.5</v>
       </c>
-      <c r="T16" s="4">
+      <c r="T16">
         <f t="shared" si="1"/>
         <v>5.7126500606536865</v>
       </c>
@@ -3010,7 +3019,7 @@
       <c r="F17">
         <v>-11.25</v>
       </c>
-      <c r="G17" s="4">
+      <c r="G17">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
@@ -3044,7 +3053,7 @@
       <c r="S17">
         <v>-11.75</v>
       </c>
-      <c r="T17" s="4">
+      <c r="T17">
         <f t="shared" si="1"/>
         <v>5.0532901287078857</v>
       </c>
@@ -3081,7 +3090,7 @@
       <c r="F18">
         <v>-9</v>
       </c>
-      <c r="G18" s="4">
+      <c r="G18">
         <f t="shared" si="0"/>
         <v>10.467299938201904</v>
       </c>
@@ -3109,7 +3118,7 @@
       <c r="S18">
         <v>-10.5</v>
       </c>
-      <c r="T18" s="4">
+      <c r="T18">
         <f t="shared" si="1"/>
         <v>22.146010160446167</v>
       </c>
@@ -3140,7 +3149,7 @@
       <c r="F19">
         <v>-13</v>
       </c>
-      <c r="G19" s="4">
+      <c r="G19">
         <f t="shared" si="0"/>
         <v>17.636569976806641</v>
       </c>
@@ -3174,7 +3183,7 @@
       <c r="S19">
         <v>-9</v>
       </c>
-      <c r="T19" s="4">
+      <c r="T19">
         <f t="shared" si="1"/>
         <v>23.3610999584198</v>
       </c>
@@ -3211,7 +3220,7 @@
       <c r="F20">
         <v>-11.5</v>
       </c>
-      <c r="G20" s="4">
+      <c r="G20">
         <f t="shared" si="0"/>
         <v>3.6116700172424316</v>
       </c>
@@ -3239,7 +3248,7 @@
       <c r="S20">
         <v>-12.5</v>
       </c>
-      <c r="T20" s="4">
+      <c r="T20">
         <f t="shared" si="1"/>
         <v>23.550359964370728</v>
       </c>
@@ -3276,7 +3285,7 @@
       <c r="F21">
         <v>-17.75</v>
       </c>
-      <c r="G21" s="4">
+      <c r="G21">
         <f t="shared" si="0"/>
         <v>2.8278200626373291</v>
       </c>
@@ -3304,7 +3313,7 @@
       <c r="S21">
         <v>-8.25</v>
       </c>
-      <c r="T21" s="4">
+      <c r="T21">
         <f t="shared" si="1"/>
         <v>14.567500114440918</v>
       </c>
@@ -3335,7 +3344,7 @@
       <c r="F22">
         <v>-17</v>
       </c>
-      <c r="G22" s="4">
+      <c r="G22">
         <f t="shared" si="0"/>
         <v>2.8819000720977783</v>
       </c>
@@ -3363,7 +3372,7 @@
       <c r="S22">
         <v>-4.5</v>
       </c>
-      <c r="T22" s="4">
+      <c r="T22">
         <f t="shared" si="1"/>
         <v>9.3723900318145752</v>
       </c>
@@ -3394,7 +3403,7 @@
       <c r="F23">
         <v>-16.25</v>
       </c>
-      <c r="G23" s="4">
+      <c r="G23">
         <f t="shared" si="0"/>
         <v>3.3792901039123535</v>
       </c>
@@ -3428,7 +3437,7 @@
       <c r="S23">
         <v>-9.75</v>
       </c>
-      <c r="T23" s="4">
+      <c r="T23">
         <f t="shared" si="1"/>
         <v>14.443419933319092</v>
       </c>
@@ -3465,7 +3474,7 @@
       <c r="F24">
         <v>-14</v>
       </c>
-      <c r="G24" s="4">
+      <c r="G24">
         <f t="shared" si="0"/>
         <v>10.740750074386597</v>
       </c>
@@ -3493,7 +3502,7 @@
       <c r="S24">
         <v>-10</v>
       </c>
-      <c r="T24" s="4">
+      <c r="T24">
         <f t="shared" si="1"/>
         <v>14.528870105743408</v>
       </c>
@@ -3524,7 +3533,7 @@
       <c r="F25">
         <v>-18.5</v>
       </c>
-      <c r="G25" s="4">
+      <c r="G25">
         <f t="shared" si="0"/>
         <v>4.6866400241851807</v>
       </c>
@@ -3558,7 +3567,7 @@
       <c r="S25">
         <v>-9.75</v>
       </c>
-      <c r="T25" s="4">
+      <c r="T25">
         <f t="shared" si="1"/>
         <v>6.9763000011444092</v>
       </c>
@@ -3595,7 +3604,7 @@
       <c r="F26">
         <v>-12.25</v>
       </c>
-      <c r="G26" s="4">
+      <c r="G26">
         <f>D26-B26</f>
         <v>10.840280055999756</v>
       </c>
@@ -3623,7 +3632,7 @@
       <c r="S26">
         <v>-13.5</v>
       </c>
-      <c r="T26" s="4">
+      <c r="T26">
         <f t="shared" si="1"/>
         <v>26.338119983673096</v>
       </c>
@@ -3654,7 +3663,7 @@
       <c r="F27">
         <v>-12.25</v>
       </c>
-      <c r="G27" s="4">
+      <c r="G27">
         <f t="shared" si="0"/>
         <v>2.810499906539917</v>
       </c>
@@ -3682,7 +3691,7 @@
       <c r="S27">
         <v>-9.5</v>
       </c>
-      <c r="T27" s="4">
+      <c r="T27">
         <f t="shared" si="1"/>
         <v>14.700200080871582</v>
       </c>
@@ -3713,7 +3722,7 @@
       <c r="F28">
         <v>-4.25</v>
       </c>
-      <c r="G28" s="4">
+      <c r="G28">
         <f t="shared" si="0"/>
         <v>17.789190053939819</v>
       </c>
@@ -3747,7 +3756,7 @@
       <c r="S28">
         <v>-14.25</v>
       </c>
-      <c r="T28" s="4">
+      <c r="T28">
         <f t="shared" si="1"/>
         <v>15.704370021820068</v>
       </c>
@@ -3784,7 +3793,7 @@
       <c r="F29">
         <v>-2</v>
       </c>
-      <c r="G29" s="4">
+      <c r="G29">
         <f t="shared" si="0"/>
         <v>10.744469881057739</v>
       </c>
@@ -3812,7 +3821,7 @@
       <c r="S29">
         <v>-14.25</v>
       </c>
-      <c r="T29" s="4">
+      <c r="T29">
         <f t="shared" si="1"/>
         <v>14.470459938049316</v>
       </c>
@@ -3843,7 +3852,7 @@
       <c r="F30">
         <v>-3</v>
       </c>
-      <c r="G30" s="4">
+      <c r="G30">
         <f t="shared" si="0"/>
         <v>17.322119951248169</v>
       </c>
@@ -3877,7 +3886,7 @@
       <c r="S30">
         <v>-10</v>
       </c>
-      <c r="T30" s="4">
+      <c r="T30">
         <f t="shared" si="1"/>
         <v>20.96068000793457</v>
       </c>
@@ -3914,7 +3923,7 @@
       <c r="F31">
         <v>-4</v>
       </c>
-      <c r="G31" s="4">
+      <c r="G31">
         <f t="shared" si="0"/>
         <v>17.713920116424561</v>
       </c>
@@ -3948,7 +3957,7 @@
       <c r="S31">
         <v>-10</v>
       </c>
-      <c r="T31" s="4">
+      <c r="T31">
         <f t="shared" si="1"/>
         <v>5.4530200958251953</v>
       </c>
@@ -3986,7 +3995,7 @@
       <c r="S32">
         <v>-9</v>
       </c>
-      <c r="T32" s="4">
+      <c r="T32">
         <f t="shared" si="1"/>
         <v>3.9217500686645508</v>
       </c>
@@ -4005,16 +4014,16 @@
       <c r="AA32" s="1"/>
     </row>
     <row r="33" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="A33" s="5" t="s">
+      <c r="A33" s="4" t="s">
         <v>317</v>
       </c>
-      <c r="B33" s="6" t="s">
+      <c r="B33" s="5" t="s">
         <v>318</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="C33" s="4" t="s">
         <v>319</v>
       </c>
-      <c r="D33" s="5" t="s">
+      <c r="D33" s="4" t="s">
         <v>320</v>
       </c>
       <c r="I33">
@@ -4041,7 +4050,7 @@
       <c r="S33">
         <v>-16.5</v>
       </c>
-      <c r="T33" s="4">
+      <c r="T33">
         <f t="shared" si="1"/>
         <v>23.838540077209473</v>
       </c>
@@ -4094,7 +4103,7 @@
       <c r="S34">
         <v>-10.25</v>
       </c>
-      <c r="T34" s="4">
+      <c r="T34">
         <f t="shared" si="1"/>
         <v>22.112809896469116</v>
       </c>
@@ -4138,7 +4147,7 @@
       <c r="S35">
         <v>-10.75</v>
       </c>
-      <c r="T35" s="4">
+      <c r="T35">
         <f t="shared" si="1"/>
         <v>14.325230121612549</v>
       </c>
@@ -4182,7 +4191,7 @@
       <c r="S36">
         <v>-14.5</v>
       </c>
-      <c r="T36" s="4">
+      <c r="T36">
         <f t="shared" si="1"/>
         <v>24.898430109024048</v>
       </c>
@@ -4220,7 +4229,7 @@
       <c r="S37">
         <v>-7.75</v>
       </c>
-      <c r="T37" s="4">
+      <c r="T37">
         <f t="shared" si="1"/>
         <v>23.728950023651123</v>
       </c>
@@ -4257,7 +4266,7 @@
       <c r="S38">
         <v>-6.75</v>
       </c>
-      <c r="T38" s="4">
+      <c r="T38">
         <f t="shared" si="1"/>
         <v>13.747260093688965</v>
       </c>
@@ -4295,7 +4304,7 @@
       <c r="S39">
         <v>-6.25</v>
       </c>
-      <c r="T39" s="4">
+      <c r="T39">
         <f t="shared" si="1"/>
         <v>5.3701798915863037</v>
       </c>
@@ -4339,7 +4348,7 @@
       <c r="S40">
         <v>-11.75</v>
       </c>
-      <c r="T40" s="4">
+      <c r="T40">
         <f t="shared" si="1"/>
         <v>12.443050146102905</v>
       </c>
@@ -4377,7 +4386,7 @@
       <c r="S41">
         <v>-16</v>
       </c>
-      <c r="T41" s="4">
+      <c r="T41">
         <f t="shared" si="1"/>
         <v>13.473690032958984</v>
       </c>
@@ -4427,7 +4436,7 @@
       <c r="S42">
         <v>-19.25</v>
       </c>
-      <c r="T42" s="4">
+      <c r="T42">
         <f t="shared" si="1"/>
         <v>24.566849946975708</v>
       </c>
@@ -4471,7 +4480,7 @@
       <c r="S43">
         <v>-17.5</v>
       </c>
-      <c r="T43" s="4">
+      <c r="T43">
         <f t="shared" si="1"/>
         <v>25.290160179138184</v>
       </c>
@@ -4509,7 +4518,7 @@
       <c r="S44">
         <v>-9.25</v>
       </c>
-      <c r="T44" s="4">
+      <c r="T44">
         <f t="shared" si="1"/>
         <v>10.092239856719971</v>
       </c>
@@ -4559,7 +4568,7 @@
       <c r="S45">
         <v>-9.5</v>
       </c>
-      <c r="T45" s="4">
+      <c r="T45">
         <f t="shared" si="1"/>
         <v>16.523210048675537</v>
       </c>
@@ -4596,7 +4605,7 @@
       <c r="S46">
         <v>-10</v>
       </c>
-      <c r="T46" s="4">
+      <c r="T46">
         <f t="shared" si="1"/>
         <v>13.920180082321167</v>
       </c>
@@ -4640,7 +4649,7 @@
       <c r="S47">
         <v>-10.25</v>
       </c>
-      <c r="T47" s="4">
+      <c r="T47">
         <f t="shared" si="1"/>
         <v>4.4875500202178955</v>
       </c>
@@ -4678,7 +4687,7 @@
       <c r="S48">
         <v>-14.25</v>
       </c>
-      <c r="T48" s="4">
+      <c r="T48">
         <f t="shared" si="1"/>
         <v>11.316580057144165</v>
       </c>
@@ -4728,7 +4737,7 @@
       <c r="S49">
         <v>-11.75</v>
       </c>
-      <c r="T49" s="4">
+      <c r="T49">
         <f t="shared" si="1"/>
         <v>25.646070003509521</v>
       </c>
@@ -4766,7 +4775,7 @@
       <c r="S50">
         <v>-10</v>
       </c>
-      <c r="T50" s="4">
+      <c r="T50">
         <f t="shared" si="1"/>
         <v>4.4551200866699219</v>
       </c>
@@ -4816,7 +4825,7 @@
       <c r="S51">
         <v>-11.75</v>
       </c>
-      <c r="T51" s="4">
+      <c r="T51">
         <f t="shared" si="1"/>
         <v>5.0824201107025146</v>
       </c>
@@ -4854,7 +4863,7 @@
       <c r="S52">
         <v>-15</v>
       </c>
-      <c r="T52" s="4">
+      <c r="T52">
         <f t="shared" si="1"/>
         <v>23.758669853210449</v>
       </c>
@@ -4898,7 +4907,7 @@
       <c r="S53">
         <v>-14</v>
       </c>
-      <c r="T53" s="4">
+      <c r="T53">
         <f t="shared" si="1"/>
         <v>14.990509986877441</v>
       </c>
@@ -4942,7 +4951,7 @@
       <c r="S54">
         <v>-15.25</v>
       </c>
-      <c r="T54" s="4">
+      <c r="T54">
         <f t="shared" si="1"/>
         <v>5.0503602027893066</v>
       </c>
@@ -4986,7 +4995,7 @@
       <c r="S55">
         <v>-13</v>
       </c>
-      <c r="T55" s="4">
+      <c r="T55">
         <f t="shared" si="1"/>
         <v>16.541189908981323</v>
       </c>
@@ -5024,7 +5033,7 @@
       <c r="S56">
         <v>-11.5</v>
       </c>
-      <c r="T56" s="4">
+      <c r="T56">
         <f t="shared" si="1"/>
         <v>29.790159940719604</v>
       </c>
@@ -5074,7 +5083,7 @@
       <c r="S57">
         <v>-11.75</v>
       </c>
-      <c r="T57" s="4">
+      <c r="T57">
         <f t="shared" si="1"/>
         <v>5.149399995803833</v>
       </c>
@@ -5118,7 +5127,7 @@
       <c r="S58">
         <v>-15.75</v>
       </c>
-      <c r="T58" s="4">
+      <c r="T58">
         <f t="shared" si="1"/>
         <v>12.685470104217529</v>
       </c>
@@ -5168,7 +5177,7 @@
       <c r="S59">
         <v>-13.25</v>
       </c>
-      <c r="T59" s="4">
+      <c r="T59">
         <f t="shared" si="1"/>
         <v>31.235309839248657</v>
       </c>
@@ -5206,7 +5215,7 @@
       <c r="S60">
         <v>-17.75</v>
       </c>
-      <c r="T60" s="4">
+      <c r="T60">
         <f t="shared" si="1"/>
         <v>33.296339988708496</v>
       </c>
@@ -5250,7 +5259,7 @@
       <c r="S61">
         <v>-17.5</v>
       </c>
-      <c r="T61" s="4">
+      <c r="T61">
         <f t="shared" si="1"/>
         <v>6.7184100151062012</v>
       </c>
@@ -5294,7 +5303,7 @@
       <c r="S62">
         <v>-10.25</v>
       </c>
-      <c r="T62" s="4">
+      <c r="T62">
         <f t="shared" si="1"/>
         <v>26.780019998550415</v>
       </c>
@@ -5338,7 +5347,7 @@
       <c r="S63">
         <v>-10.75</v>
       </c>
-      <c r="T63" s="4">
+      <c r="T63">
         <f t="shared" si="1"/>
         <v>33.397599935531616</v>
       </c>
@@ -5381,7 +5390,7 @@
       <c r="S64">
         <v>-10.5</v>
       </c>
-      <c r="T64" s="4">
+      <c r="T64">
         <f t="shared" si="1"/>
         <v>3.2853400707244873</v>
       </c>
@@ -5419,7 +5428,7 @@
       <c r="S65">
         <v>-15</v>
       </c>
-      <c r="T65" s="4">
+      <c r="T65">
         <f t="shared" si="1"/>
         <v>15.155380010604858</v>
       </c>
@@ -5463,7 +5472,7 @@
       <c r="S66">
         <v>-11.25</v>
       </c>
-      <c r="T66" s="4">
+      <c r="T66">
         <f t="shared" si="1"/>
         <v>4.4371399879455566</v>
       </c>
@@ -5513,7 +5522,7 @@
       <c r="S67">
         <v>-13</v>
       </c>
-      <c r="T67" s="4">
+      <c r="T67">
         <f t="shared" ref="T67:T79" si="2">Q67-O67</f>
         <v>15.845779895782471</v>
       </c>
@@ -5556,7 +5565,7 @@
       <c r="S68">
         <v>-17.5</v>
       </c>
-      <c r="T68" s="4">
+      <c r="T68">
         <f t="shared" si="2"/>
         <v>13.347949981689453</v>
       </c>
@@ -5600,7 +5609,7 @@
       <c r="S69">
         <v>-9.75</v>
       </c>
-      <c r="T69" s="4">
+      <c r="T69">
         <f t="shared" si="2"/>
         <v>5.4510500431060791</v>
       </c>
@@ -5638,7 +5647,7 @@
       <c r="S70">
         <v>-16</v>
       </c>
-      <c r="T70" s="4">
+      <c r="T70">
         <f t="shared" si="2"/>
         <v>25.006319999694824</v>
       </c>
@@ -5688,7 +5697,7 @@
       <c r="S71">
         <v>-13.25</v>
       </c>
-      <c r="T71" s="4">
+      <c r="T71">
         <f t="shared" si="2"/>
         <v>24.74702000617981</v>
       </c>
@@ -5726,7 +5735,7 @@
       <c r="S72">
         <v>-18.5</v>
       </c>
-      <c r="T72" s="4">
+      <c r="T72">
         <f t="shared" si="2"/>
         <v>16.368160009384155</v>
       </c>
@@ -5770,7 +5779,7 @@
       <c r="S73">
         <v>-16.75</v>
       </c>
-      <c r="T73" s="4">
+      <c r="T73">
         <f t="shared" si="2"/>
         <v>25.202349901199341</v>
       </c>
@@ -5808,7 +5817,7 @@
       <c r="S74">
         <v>-15.25</v>
       </c>
-      <c r="T74" s="4">
+      <c r="T74">
         <f t="shared" si="2"/>
         <v>5.5362699031829834</v>
       </c>
@@ -5851,7 +5860,7 @@
       <c r="S75">
         <v>-14.5</v>
       </c>
-      <c r="T75" s="4">
+      <c r="T75">
         <f t="shared" si="2"/>
         <v>16.946410179138184</v>
       </c>
@@ -5889,7 +5898,7 @@
       <c r="S76">
         <v>-17</v>
       </c>
-      <c r="T76" s="4">
+      <c r="T76">
         <f t="shared" si="2"/>
         <v>4.0722601413726807</v>
       </c>
@@ -5933,7 +5942,7 @@
       <c r="S77">
         <v>-10.5</v>
       </c>
-      <c r="T77" s="4">
+      <c r="T77">
         <f t="shared" si="2"/>
         <v>3.7019798755645752</v>
       </c>
@@ -5971,7 +5980,7 @@
       <c r="S78">
         <v>-13</v>
       </c>
-      <c r="T78" s="4">
+      <c r="T78">
         <f t="shared" si="2"/>
         <v>30.015379905700684</v>
       </c>
@@ -6015,7 +6024,7 @@
       <c r="S79">
         <v>-15</v>
       </c>
-      <c r="T79" s="4">
+      <c r="T79">
         <f t="shared" si="2"/>
         <v>5.6877601146697998</v>
       </c>
@@ -7107,24 +7116,24 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>321</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>317</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>318</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>324</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="4" t="s">
         <v>320</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="4" t="s">
         <v>322</v>
       </c>
       <c r="B2">
@@ -7145,22 +7154,22 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="4" t="s">
         <v>323</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="6">
         <f>(COUNT(all!N2:N79)/300)*100</f>
         <v>26</v>
       </c>
-      <c r="C3" s="11">
+      <c r="C3" s="9">
         <f>AVERAGE(all!T2:T79)</f>
         <v>15.022215528365892</v>
       </c>
-      <c r="D3" s="7" cm="1">
+      <c r="D3" s="6" cm="1">
         <f t="array" ref="D3">SUMPRODUCT(--( COUNTIF(all!V2:V99,all!P2:P79)&gt;0))</f>
         <v>53</v>
       </c>
-      <c r="E3" s="7">
+      <c r="E3" s="6">
         <f>(D3/COUNT(all!N2:N79))*100</f>
         <v>67.948717948717956</v>
       </c>

</xml_diff>